<commit_message>
feat: expand metafiction and add autofiction genres
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -4067,7 +4067,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z40" t="str">
-        <v>Essays</v>
+        <v>essays, autofiction, metafiction</v>
       </c>
       <c r="AA40" t="str">
         <v>France</v>
@@ -6735,7 +6735,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z69" t="str">
-        <v>Literary Fiction</v>
+        <v>literary fiction, metafiction</v>
       </c>
       <c r="AA69" t="str">
         <v>United States</v>
@@ -8115,7 +8115,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z84" t="str">
-        <v>Fantasy, Classics</v>
+        <v>fantasy, classics, metafiction</v>
       </c>
       <c r="AA84" t="str">
         <v>Italy</v>
@@ -16303,7 +16303,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z173" t="str">
-        <v>Literary Fiction, Classics</v>
+        <v>literary fiction, classics, metafiction</v>
       </c>
       <c r="AA173" t="str">
         <v>United Kingdom</v>
@@ -21639,7 +21639,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z231" t="str">
-        <v>Science Fiction, War, Classics</v>
+        <v>science fiction, war, classics, metafiction</v>
       </c>
       <c r="AA231" t="str">
         <v>United States</v>
@@ -26147,7 +26147,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z280" t="str">
-        <v>science fiction, humor, classics, absurdism</v>
+        <v>science fiction, humor, classics, absurdism, metafiction</v>
       </c>
       <c r="AA280" t="str">
         <v>United States</v>
@@ -37923,7 +37923,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z408" t="str">
-        <v>literary fiction, satire, picaresque</v>
+        <v>literary fiction, satire, picaresque, metafiction</v>
       </c>
       <c r="AA408" t="str">
         <v>Brazil</v>
@@ -49515,7 +49515,7 @@
         <v>Non-Fiction</v>
       </c>
       <c r="Z534" t="str">
-        <v>Biography</v>
+        <v>biography, autofiction, metafiction</v>
       </c>
       <c r="AA534" t="str">
         <v>United States</v>
@@ -52827,7 +52827,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z570" t="str">
-        <v>Magical Realism, Historical Fiction</v>
+        <v>magical realism, historical fiction, metafiction</v>
       </c>
       <c r="AA570" t="str">
         <v>India</v>
@@ -53011,7 +53011,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z572" t="str">
-        <v>Historical Fiction, Mystery, Classics</v>
+        <v>historical fiction, mystery, classics, metafiction</v>
       </c>
       <c r="AA572" t="str">
         <v>Italy</v>
@@ -57243,7 +57243,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z618" t="str">
-        <v>Historical Fiction, Mystery</v>
+        <v>historical fiction, mystery, metafiction</v>
       </c>
       <c r="AA618" t="str">
         <v>Canada</v>

</xml_diff>

<commit_message>
chore: update shelf + Goodreads data so newly published reviews link
Reflects the current book export/shelf state (incl. the reviews published
in the previous commit) so the /book-reviews shelf marks them clickable.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGGTHD9uZpyHh8EVS3UX2k
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD713"/>
+  <dimension ref="A1:AD717"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -46031,7 +46031,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1537315266i/40163119.jpg</v>
       </c>
       <c r="AD496" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="497">
@@ -49435,7 +49435,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1414608893i/2715.jpg</v>
       </c>
       <c r="AD533" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="534">
@@ -58359,7 +58359,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1389164885i/846101.jpg</v>
       </c>
       <c r="AD630" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="631">
@@ -62683,7 +62683,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1327364614i/3115359.jpg</v>
       </c>
       <c r="AD677" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="678">
@@ -63876,10 +63876,10 @@
         <v>English</v>
       </c>
       <c r="AC690" t="str">
-        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1728768241i/17332218.jpg</v>
+        <v>https://images-na.ssl-images-amazon.com/images/P/0765326361.01.L.jpg</v>
       </c>
       <c r="AD690" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="691">
@@ -64155,7 +64155,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1654573897i/34002132.jpg</v>
       </c>
       <c r="AD693" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="694">
@@ -64799,7 +64799,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1334162378i/776459.jpg</v>
       </c>
       <c r="AD700" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="701">
@@ -64891,7 +64891,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1588260981i/1234310.jpg</v>
       </c>
       <c r="AD701" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="702">
@@ -65719,7 +65719,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1387717495i/322067.jpg</v>
       </c>
       <c r="AD710" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="711">
@@ -65946,8 +65946,8 @@
       <c r="M713">
         <v>1947</v>
       </c>
-      <c r="N713" t="str">
-        <v/>
+      <c r="N713" s="1" t="d">
+        <v>2026-06-14T00:00:00.000Z</v>
       </c>
       <c r="O713" s="1" t="d">
         <v>2026-05-23T00:00:00.000Z</v>
@@ -65959,7 +65959,7 @@
         <v>currently-reading (#1), 2026 (#21)</v>
       </c>
       <c r="R713" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S713" t="str">
         <v/>
@@ -65998,16 +65998,384 @@
         <v>Mine</v>
       </c>
     </row>
+    <row r="714">
+      <c r="A714">
+        <v>235699916</v>
+      </c>
+      <c r="B714" t="str">
+        <v>Suspicion</v>
+      </c>
+      <c r="C714" t="str">
+        <v>Seichō Matsumoto</v>
+      </c>
+      <c r="D714" t="str">
+        <v>Matsumoto, SeichÅ</v>
+      </c>
+      <c r="E714" t="str">
+        <v>Jesse Kirkwood</v>
+      </c>
+      <c r="F714" t="str">
+        <v>0593979060</v>
+      </c>
+      <c r="G714" t="str">
+        <v>9780593979068</v>
+      </c>
+      <c r="H714">
+        <v>3</v>
+      </c>
+      <c r="I714" t="str">
+        <v>Modern Library</v>
+      </c>
+      <c r="J714" t="str">
+        <v>Paperback</v>
+      </c>
+      <c r="K714">
+        <v>128</v>
+      </c>
+      <c r="L714">
+        <v>2026</v>
+      </c>
+      <c r="M714">
+        <v>1982</v>
+      </c>
+      <c r="N714" s="1" t="d">
+        <v>2026-07-01T00:00:00.000Z</v>
+      </c>
+      <c r="O714" s="1" t="d">
+        <v>2026-06-27T00:00:00.000Z</v>
+      </c>
+      <c r="P714">
+        <v>2026</v>
+      </c>
+      <c r="Q714" t="str">
+        <v>2026 (#24)</v>
+      </c>
+      <c r="R714" t="str">
+        <v>read</v>
+      </c>
+      <c r="S714" t="str">
+        <v/>
+      </c>
+      <c r="T714" t="str">
+        <v/>
+      </c>
+      <c r="U714" t="str">
+        <v/>
+      </c>
+      <c r="V714">
+        <v>1</v>
+      </c>
+      <c r="W714">
+        <v>0</v>
+      </c>
+      <c r="X714" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y714" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z714" t="str">
+        <v>Crime, Mystery</v>
+      </c>
+      <c r="AA714" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="AB714" t="str">
+        <v>Japanese</v>
+      </c>
+      <c r="AC714" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1753932733i/235699916.jpg</v>
+      </c>
+      <c r="AD714" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715">
+        <v>1697369</v>
+      </c>
+      <c r="B715" t="str">
+        <v>The Awakening</v>
+      </c>
+      <c r="C715" t="str">
+        <v>Kate Chopin</v>
+      </c>
+      <c r="D715" t="str">
+        <v>Chopin, Kate</v>
+      </c>
+      <c r="E715" t="str">
+        <v/>
+      </c>
+      <c r="F715" t="str">
+        <v>0553211943</v>
+      </c>
+      <c r="G715" t="str">
+        <v>9780553211948</v>
+      </c>
+      <c r="H715">
+        <v>3</v>
+      </c>
+      <c r="I715" t="str">
+        <v>Bantam Classics</v>
+      </c>
+      <c r="J715" t="str">
+        <v>Mass Market Paperback</v>
+      </c>
+      <c r="K715">
+        <v>205</v>
+      </c>
+      <c r="L715">
+        <v>1985</v>
+      </c>
+      <c r="M715">
+        <v>1899</v>
+      </c>
+      <c r="N715" s="1" t="d">
+        <v>2026-06-27T00:00:00.000Z</v>
+      </c>
+      <c r="O715" s="1" t="d">
+        <v>2026-05-10T00:00:00.000Z</v>
+      </c>
+      <c r="P715">
+        <v>2026</v>
+      </c>
+      <c r="Q715" t="str">
+        <v>2026 (#23)</v>
+      </c>
+      <c r="R715" t="str">
+        <v>read</v>
+      </c>
+      <c r="S715" t="str">
+        <v/>
+      </c>
+      <c r="T715" t="str">
+        <v/>
+      </c>
+      <c r="U715" t="str">
+        <v/>
+      </c>
+      <c r="V715">
+        <v>1</v>
+      </c>
+      <c r="W715">
+        <v>0</v>
+      </c>
+      <c r="X715" t="str">
+        <v>Female</v>
+      </c>
+      <c r="Y715" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z715" t="str">
+        <v>Literary Fiction, Classics</v>
+      </c>
+      <c r="AA715" t="str">
+        <v>United States</v>
+      </c>
+      <c r="AB715" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC715" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1413729933i/1697369.jpg</v>
+      </c>
+      <c r="AD715" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716">
+        <v>238226991</v>
+      </c>
+      <c r="B716" t="str">
+        <v>London Falling: A Mysterious Death in a Gilded City and a Family's Search for Truth</v>
+      </c>
+      <c r="C716" t="str">
+        <v>Patrick Radden Keefe</v>
+      </c>
+      <c r="D716" t="str">
+        <v>Keefe, Patrick Radden</v>
+      </c>
+      <c r="E716" t="str">
+        <v/>
+      </c>
+      <c r="F716" t="str">
+        <v>0385548532</v>
+      </c>
+      <c r="G716" t="str">
+        <v>9780385548533</v>
+      </c>
+      <c r="H716">
+        <v>3</v>
+      </c>
+      <c r="I716" t="str">
+        <v>Doubleday</v>
+      </c>
+      <c r="J716" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K716">
+        <v>361</v>
+      </c>
+      <c r="L716">
+        <v>2026</v>
+      </c>
+      <c r="M716">
+        <v>2026</v>
+      </c>
+      <c r="N716" s="1" t="d">
+        <v>2026-06-22T00:00:00.000Z</v>
+      </c>
+      <c r="O716" s="1" t="d">
+        <v>2026-06-03T00:00:00.000Z</v>
+      </c>
+      <c r="P716">
+        <v>2026</v>
+      </c>
+      <c r="Q716" t="str">
+        <v>2026 (#22)</v>
+      </c>
+      <c r="R716" t="str">
+        <v>read</v>
+      </c>
+      <c r="S716" t="str">
+        <v/>
+      </c>
+      <c r="T716" t="str">
+        <v/>
+      </c>
+      <c r="U716" t="str">
+        <v/>
+      </c>
+      <c r="V716">
+        <v>1</v>
+      </c>
+      <c r="W716">
+        <v>0</v>
+      </c>
+      <c r="X716" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y716" t="str">
+        <v>Non-Fiction</v>
+      </c>
+      <c r="Z716" t="str">
+        <v>True Crime, Journalism</v>
+      </c>
+      <c r="AA716" t="str">
+        <v>United States</v>
+      </c>
+      <c r="AB716" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC716" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1751942777i/238226991.jpg</v>
+      </c>
+      <c r="AD716" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717">
+        <v>247522184</v>
+      </c>
+      <c r="B717" t="str">
+        <v>Yesteryear</v>
+      </c>
+      <c r="C717" t="str">
+        <v>Caro Claire Burke</v>
+      </c>
+      <c r="D717" t="str">
+        <v>Burke, Caro Claire</v>
+      </c>
+      <c r="E717" t="str">
+        <v/>
+      </c>
+      <c r="F717" t="str">
+        <v>0008742766</v>
+      </c>
+      <c r="G717" t="str">
+        <v>9780008742768</v>
+      </c>
+      <c r="H717">
+        <v>0</v>
+      </c>
+      <c r="I717" t="str">
+        <v>Fourth Estate</v>
+      </c>
+      <c r="J717" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K717">
+        <v>391</v>
+      </c>
+      <c r="L717">
+        <v>2026</v>
+      </c>
+      <c r="M717">
+        <v>2026</v>
+      </c>
+      <c r="N717" t="str">
+        <v/>
+      </c>
+      <c r="O717" s="1" t="d">
+        <v>2026-04-19T00:00:00.000Z</v>
+      </c>
+      <c r="P717" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q717" t="str">
+        <v>currently-reading (#1), 2026 (#25)</v>
+      </c>
+      <c r="R717" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S717" t="str">
+        <v/>
+      </c>
+      <c r="T717" t="str">
+        <v/>
+      </c>
+      <c r="U717" t="str">
+        <v/>
+      </c>
+      <c r="V717">
+        <v>1</v>
+      </c>
+      <c r="W717">
+        <v>0</v>
+      </c>
+      <c r="X717" t="str">
+        <v>Female</v>
+      </c>
+      <c r="Y717" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z717" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA717" t="str">
+        <v>United States</v>
+      </c>
+      <c r="AB717" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC717" t="str">
+        <v>https://covers.openlibrary.org/b/id/15213215-L.jpg</v>
+      </c>
+      <c r="AD717" t="str">
+        <v>Claude</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD713"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD717"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A1000"/>
+  <dimension ref="A1:A47"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -66245,8 +66613,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A1000"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: shelf regen, review copy edits, blockquote + year-rail polish
Regenerate the shelf, tidy five review posts, restyle article
blockquotes into a bordered card, add per-year counts to the
book-reviews year rail, and stash the SEO roadmap notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmbiAAYYLqrgwexhWaLTBe
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -65745,7 +65745,7 @@
         <v/>
       </c>
       <c r="H711">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I711" t="str">
         <v>Pocket</v>
@@ -65929,7 +65929,7 @@
         <v/>
       </c>
       <c r="H713">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I713" t="str">
         <v/>
@@ -66087,7 +66087,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1753932733i/235699916.jpg</v>
       </c>
       <c r="AD714" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="715">

</xml_diff>

<commit_message>
data: reclassify author countries (Greek tradition; Camus → Algeria)
Nonnus of Panopolis, Lucian of Samosata, Quintus Smyrnaeus → Greece
(classified by Greek literary tradition rather than modern birthplace
geography, matching Herodotus). Albert Camus → Algeria (birthplace,
consistent with the shelf's origin convention). Edited the Country
column in website-books.xlsx and regenerated shelf.json.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmbiAAYYLqrgwexhWaLTBe
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -1862,7 +1862,7 @@
         <v>Satire</v>
       </c>
       <c r="AA16" t="str">
-        <v>Syria</v>
+        <v>Greece</v>
       </c>
       <c r="AB16" t="str">
         <v>Ancient Greek</v>
@@ -4162,7 +4162,7 @@
         <v>philosophy, classics, absurdism</v>
       </c>
       <c r="AA41" t="str">
-        <v>France</v>
+        <v>Algeria</v>
       </c>
       <c r="AB41" t="str">
         <v>French</v>
@@ -7842,7 +7842,7 @@
         <v>Philosophy</v>
       </c>
       <c r="AA81" t="str">
-        <v>France</v>
+        <v>Algeria</v>
       </c>
       <c r="AB81" t="str">
         <v>French</v>
@@ -13095,7 +13095,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1619399676i/721028.jpg</v>
       </c>
       <c r="AD138" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="139">
@@ -22010,7 +22010,7 @@
         <v>literary fiction, absurdism</v>
       </c>
       <c r="AA235" t="str">
-        <v>France</v>
+        <v>Algeria</v>
       </c>
       <c r="AB235" t="str">
         <v>French</v>
@@ -42894,7 +42894,7 @@
         <v>Mythology</v>
       </c>
       <c r="AA462" t="str">
-        <v>Turkey</v>
+        <v>Greece</v>
       </c>
       <c r="AB462" t="str">
         <v>Ancient Greek</v>
@@ -52554,7 +52554,7 @@
         <v>Epic, Poetry</v>
       </c>
       <c r="AA567" t="str">
-        <v>Egypt</v>
+        <v>Greece</v>
       </c>
       <c r="AB567" t="str">
         <v>Ancient Greek</v>
@@ -54854,7 +54854,7 @@
         <v>Epic, Poetry</v>
       </c>
       <c r="AA592" t="str">
-        <v>Egypt</v>
+        <v>Greece</v>
       </c>
       <c r="AB592" t="str">
         <v>Ancient Greek</v>
@@ -55498,7 +55498,7 @@
         <v>Epic, Poetry</v>
       </c>
       <c r="AA599" t="str">
-        <v>Egypt</v>
+        <v>Greece</v>
       </c>
       <c r="AB599" t="str">
         <v>Ancient Greek</v>
@@ -60383,7 +60383,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1523897945i/36454667.jpg</v>
       </c>
       <c r="AD652" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="653">
@@ -66271,7 +66271,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1751942777i/238226991.jpg</v>
       </c>
       <c r="AD716" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="717">

</xml_diff>

<commit_message>
data: Meditations original language Latin → Ancient Greek
Marcus Aurelius wrote the Meditations in Koine Greek; country stays Italy
(he was Roman).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmbiAAYYLqrgwexhWaLTBe
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -26061,7 +26061,7 @@
         <v>Italy</v>
       </c>
       <c r="AB279" t="str">
-        <v>Latin</v>
+        <v>Ancient Greek</v>
       </c>
       <c r="AC279" t="str">
         <v>https://images-na.ssl-images-amazon.com/images/P/0140449337.01.L.jpg</v>
@@ -26245,7 +26245,7 @@
         <v>Italy</v>
       </c>
       <c r="AB281" t="str">
-        <v>Latin</v>
+        <v>Ancient Greek</v>
       </c>
       <c r="AC281" t="str">
         <v>https://images-na.ssl-images-amazon.com/images/P/0140449337.01.L.jpg</v>

</xml_diff>

<commit_message>
data: tag Taiwan Travelogue + Salt with Food genre
Extend the existing Food genre to two books that highlight recipes:
Taiwan Travelogue (Literary Fiction) and Salt: A World History
(History, Kurlansky's embedded period recipes). Regenerated shelf.json.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmbiAAYYLqrgwexhWaLTBe
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -25779,7 +25779,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z276" t="str">
-        <v>Literary Fiction</v>
+        <v>Literary Fiction, Food</v>
       </c>
       <c r="AA276" t="str">
         <v>Taiwan</v>
@@ -49423,7 +49423,7 @@
         <v>non-Fiction</v>
       </c>
       <c r="Z533" t="str">
-        <v>History</v>
+        <v>History, Food</v>
       </c>
       <c r="AA533" t="str">
         <v>United States</v>
@@ -65811,7 +65811,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1287080489i/729728.jpg</v>
       </c>
       <c r="AD711" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="712">
@@ -65903,7 +65903,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1332036031i/299758.jpg</v>
       </c>
       <c r="AD712" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="713">

</xml_diff>

<commit_message>
data: import latest Goodreads export, publish Yesteryear review
Adds The Frolic of the Beasts (finished) and Ways of Seeing (currently
reading), regenerates shelf data, and publishes the Yesteryear review.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgXGhm4Nq3drSQQrLtkp8N
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD721"/>
+  <dimension ref="A1:AD722"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -66389,7 +66389,7 @@
         <v>9780525434153</v>
       </c>
       <c r="H718">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I718" t="str">
         <v>Vintage</v>
@@ -66406,8 +66406,8 @@
       <c r="M718">
         <v>1961</v>
       </c>
-      <c r="N718" t="str">
-        <v/>
+      <c r="N718" s="1" t="d">
+        <v>2026-07-15T00:00:00.000Z</v>
       </c>
       <c r="O718" s="1" t="d">
         <v>2026-05-23T00:00:00.000Z</v>
@@ -66419,7 +66419,7 @@
         <v>currently-reading (#1), 2026 (#26)</v>
       </c>
       <c r="R718" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S718" t="str">
         <v/>
@@ -66734,9 +66734,101 @@
         <v>Claude</v>
       </c>
     </row>
+    <row r="722">
+      <c r="A722">
+        <v>2784</v>
+      </c>
+      <c r="B722" t="str">
+        <v>Ways of Seeing</v>
+      </c>
+      <c r="C722" t="str">
+        <v>John Berger</v>
+      </c>
+      <c r="D722" t="str">
+        <v>Berger, John</v>
+      </c>
+      <c r="E722" t="str">
+        <v/>
+      </c>
+      <c r="F722" t="str">
+        <v>0140135154</v>
+      </c>
+      <c r="G722" t="str">
+        <v>9780140135152</v>
+      </c>
+      <c r="H722">
+        <v>0</v>
+      </c>
+      <c r="I722" t="str">
+        <v>Penguin</v>
+      </c>
+      <c r="J722" t="str">
+        <v>Paperback</v>
+      </c>
+      <c r="K722">
+        <v>176</v>
+      </c>
+      <c r="L722">
+        <v>1990</v>
+      </c>
+      <c r="M722">
+        <v>1972</v>
+      </c>
+      <c r="N722" t="str">
+        <v/>
+      </c>
+      <c r="O722" s="1" t="d">
+        <v>2026-04-13T00:00:00.000Z</v>
+      </c>
+      <c r="P722" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q722" t="str">
+        <v>currently-reading (#1), 2026 (#27)</v>
+      </c>
+      <c r="R722" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S722" t="str">
+        <v/>
+      </c>
+      <c r="T722" t="str">
+        <v/>
+      </c>
+      <c r="U722" t="str">
+        <v/>
+      </c>
+      <c r="V722">
+        <v>1</v>
+      </c>
+      <c r="W722">
+        <v>0</v>
+      </c>
+      <c r="X722" t="str">
+        <v/>
+      </c>
+      <c r="Y722" t="str">
+        <v/>
+      </c>
+      <c r="Z722" t="str">
+        <v/>
+      </c>
+      <c r="AA722" t="str">
+        <v/>
+      </c>
+      <c r="AB722" t="str">
+        <v/>
+      </c>
+      <c r="AC722" t="str">
+        <v>https://covers.openlibrary.org/b/isbn/9780140135152-L.jpg?default=false</v>
+      </c>
+      <c r="AD722" t="str">
+        <v>Claude</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD721"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD722"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
data: set custom cover for Ways of Seeing
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgXGhm4Nq3drSQQrLtkp8N
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -66363,7 +66363,7 @@
         <v>https://covers.openlibrary.org/b/id/15213215-L.jpg</v>
       </c>
       <c r="AD717" t="str">
-        <v>Claude</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="718">
@@ -66499,7 +66499,7 @@
         <v>1890</v>
       </c>
       <c r="N719" s="1" t="d">
-        <v>2014-02-27T19:00:00.000Z</v>
+        <v>2014-02-27T18:59:59.999Z</v>
       </c>
       <c r="O719" s="1" t="d">
         <v>2026-07-11T00:00:00.000Z</v>
@@ -66820,10 +66820,10 @@
         <v/>
       </c>
       <c r="AC722" t="str">
-        <v>https://covers.openlibrary.org/b/isbn/9780140135152-L.jpg?default=false</v>
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1703328414i/2784.jpg</v>
       </c>
       <c r="AD722" t="str">
-        <v>Claude</v>
+        <v>Mine</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: import latest Goodreads export, add Bolaño/Lispector reads
Adds The Passion According to G.H. (finished) and The Savage
Detectives (currently reading), marks Ways of Seeing as read, and
sets custom covers for all three.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD722"/>
+  <dimension ref="A1:AD724"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -66757,7 +66757,7 @@
         <v>9780140135152</v>
       </c>
       <c r="H722">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I722" t="str">
         <v>Penguin</v>
@@ -66774,8 +66774,8 @@
       <c r="M722">
         <v>1972</v>
       </c>
-      <c r="N722" t="str">
-        <v/>
+      <c r="N722" s="1" t="d">
+        <v>2026-07-16T00:00:00.000Z</v>
       </c>
       <c r="O722" s="1" t="d">
         <v>2026-04-13T00:00:00.000Z</v>
@@ -66787,7 +66787,7 @@
         <v>currently-reading (#1), 2026 (#27)</v>
       </c>
       <c r="R722" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S722" t="str">
         <v/>
@@ -66805,19 +66805,19 @@
         <v>0</v>
       </c>
       <c r="X722" t="str">
-        <v/>
+        <v>Male</v>
       </c>
       <c r="Y722" t="str">
-        <v/>
+        <v>Nonfiction</v>
       </c>
       <c r="Z722" t="str">
-        <v/>
+        <v>Art Criticism</v>
       </c>
       <c r="AA722" t="str">
-        <v/>
+        <v>UK</v>
       </c>
       <c r="AB722" t="str">
-        <v/>
+        <v>English</v>
       </c>
       <c r="AC722" t="str">
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1703328414i/2784.jpg</v>
@@ -66826,9 +66826,193 @@
         <v>Mine</v>
       </c>
     </row>
+    <row r="723">
+      <c r="A723">
+        <v>13082436</v>
+      </c>
+      <c r="B723" t="str">
+        <v>The Passion According to G.H.</v>
+      </c>
+      <c r="C723" t="str">
+        <v>Clarice Lispector</v>
+      </c>
+      <c r="D723" t="str">
+        <v>Lispector, Clarice</v>
+      </c>
+      <c r="E723" t="str">
+        <v>Idra Novey, Caetano Veloso, Benjamin Moser</v>
+      </c>
+      <c r="F723" t="str">
+        <v>0811219682</v>
+      </c>
+      <c r="G723" t="str">
+        <v>9780811219686</v>
+      </c>
+      <c r="H723">
+        <v>3</v>
+      </c>
+      <c r="I723" t="str">
+        <v>New Directions</v>
+      </c>
+      <c r="J723" t="str">
+        <v>Paperback</v>
+      </c>
+      <c r="K723">
+        <v>193</v>
+      </c>
+      <c r="L723">
+        <v>2012</v>
+      </c>
+      <c r="M723">
+        <v>1964</v>
+      </c>
+      <c r="N723" s="1" t="d">
+        <v>2026-07-21T00:00:00.000Z</v>
+      </c>
+      <c r="O723" s="1" t="d">
+        <v>2026-04-24T00:00:00.000Z</v>
+      </c>
+      <c r="P723">
+        <v>2026</v>
+      </c>
+      <c r="Q723" t="str">
+        <v>2026 (#28)</v>
+      </c>
+      <c r="R723" t="str">
+        <v>read</v>
+      </c>
+      <c r="S723" t="str">
+        <v/>
+      </c>
+      <c r="T723" t="str">
+        <v/>
+      </c>
+      <c r="U723" t="str">
+        <v/>
+      </c>
+      <c r="V723">
+        <v>1</v>
+      </c>
+      <c r="W723">
+        <v>0</v>
+      </c>
+      <c r="X723" t="str">
+        <v>Female</v>
+      </c>
+      <c r="Y723" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z723" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA723" t="str">
+        <v>Brazil</v>
+      </c>
+      <c r="AB723" t="str">
+        <v>Portuguese</v>
+      </c>
+      <c r="AC723" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1655722528i/13082436.jpg</v>
+      </c>
+      <c r="AD723" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724">
+        <v>63033</v>
+      </c>
+      <c r="B724" t="str">
+        <v>The Savage Detectives</v>
+      </c>
+      <c r="C724" t="str">
+        <v>Roberto Bolaño</v>
+      </c>
+      <c r="D724" t="str">
+        <v>Bolaño, Roberto</v>
+      </c>
+      <c r="E724" t="str">
+        <v>Natasha Wimmer</v>
+      </c>
+      <c r="F724" t="str">
+        <v>0374191484</v>
+      </c>
+      <c r="G724" t="str">
+        <v>9780374191481</v>
+      </c>
+      <c r="H724">
+        <v>0</v>
+      </c>
+      <c r="I724" t="str">
+        <v>Farrar, Straus and Giroux</v>
+      </c>
+      <c r="J724" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K724">
+        <v>577</v>
+      </c>
+      <c r="L724">
+        <v>2007</v>
+      </c>
+      <c r="M724">
+        <v>1998</v>
+      </c>
+      <c r="N724" t="str">
+        <v/>
+      </c>
+      <c r="O724" s="1" t="d">
+        <v>2026-05-27T00:00:00.000Z</v>
+      </c>
+      <c r="P724" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q724" t="str">
+        <v>currently-reading (#1), 2026 (#29)</v>
+      </c>
+      <c r="R724" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S724" t="str">
+        <v/>
+      </c>
+      <c r="T724" t="str">
+        <v/>
+      </c>
+      <c r="U724" t="str">
+        <v/>
+      </c>
+      <c r="V724">
+        <v>1</v>
+      </c>
+      <c r="W724">
+        <v>0</v>
+      </c>
+      <c r="X724" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y724" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z724" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA724" t="str">
+        <v>Chile</v>
+      </c>
+      <c r="AB724" t="str">
+        <v>Spanish</v>
+      </c>
+      <c r="AC724" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1342651149i/63033.jpg</v>
+      </c>
+      <c r="AD724" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD722"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD724"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
content: publish The Savage Detectives review, sync Goodreads import
- Publish full review of The Savage Detectives with Sión poem image
- Import latest Goodreads export: The Devotion of Suspect X finished,
  The Blacktongue Thief now currently-reading
- Strip series suffix (e.g. "(Series, #1)") from currently-reading titles
- Add cover URLs for Suspect X, Steppenwolf, and Savage Detectives stubs

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD724"/>
+  <dimension ref="A1:AD727"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23675,7 +23675,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1348020113i/9618464.jpg</v>
       </c>
       <c r="AD253" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="254">
@@ -40353,7 +40353,7 @@
         <v/>
       </c>
       <c r="H435">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I435" t="str">
         <v>Naulit Publishing House</v>
@@ -65745,7 +65745,7 @@
         <v/>
       </c>
       <c r="H711">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I711" t="str">
         <v>Pocket</v>
@@ -66179,7 +66179,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1413729933i/1697369.jpg</v>
       </c>
       <c r="AD715" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="716">
@@ -66455,7 +66455,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1513997033i/35952941.jpg</v>
       </c>
       <c r="AD718" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="719">
@@ -66823,7 +66823,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1703328414i/2784.jpg</v>
       </c>
       <c r="AD722" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="723">
@@ -66915,7 +66915,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1655722528i/13082436.jpg</v>
       </c>
       <c r="AD723" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="724">
@@ -66941,7 +66941,7 @@
         <v>9780374191481</v>
       </c>
       <c r="H724">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I724" t="str">
         <v>Farrar, Straus and Giroux</v>
@@ -66958,8 +66958,8 @@
       <c r="M724">
         <v>1998</v>
       </c>
-      <c r="N724" t="str">
-        <v/>
+      <c r="N724" s="1" t="d">
+        <v>2026-08-08T00:00:00.000Z</v>
       </c>
       <c r="O724" s="1" t="d">
         <v>2026-05-27T00:00:00.000Z</v>
@@ -66971,7 +66971,7 @@
         <v>currently-reading (#1), 2026 (#29)</v>
       </c>
       <c r="R724" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S724" t="str">
         <v/>
@@ -67010,9 +67010,285 @@
         <v>Mine</v>
       </c>
     </row>
+    <row r="725">
+      <c r="A725">
+        <v>69819</v>
+      </c>
+      <c r="B725" t="str">
+        <v>Steppenwolf</v>
+      </c>
+      <c r="C725" t="str">
+        <v>Hermann Hesse</v>
+      </c>
+      <c r="D725" t="str">
+        <v>Hesse, Hermann</v>
+      </c>
+      <c r="E725" t="str">
+        <v/>
+      </c>
+      <c r="F725" t="str">
+        <v>0553131745</v>
+      </c>
+      <c r="G725" t="str">
+        <v>9780553131741</v>
+      </c>
+      <c r="H725">
+        <v>4</v>
+      </c>
+      <c r="I725" t="str">
+        <v>Bantam Books, Inc.</v>
+      </c>
+      <c r="J725" t="str">
+        <v>Mass Market Paperback</v>
+      </c>
+      <c r="K725">
+        <v>248</v>
+      </c>
+      <c r="L725">
+        <v>1979</v>
+      </c>
+      <c r="M725">
+        <v>1927</v>
+      </c>
+      <c r="N725" s="1" t="d">
+        <v>2026-08-10T00:00:00.000Z</v>
+      </c>
+      <c r="O725" s="1" t="d">
+        <v>2023-11-05T00:00:00.000Z</v>
+      </c>
+      <c r="P725">
+        <v>2026</v>
+      </c>
+      <c r="Q725" t="str">
+        <v>2026 (#30)</v>
+      </c>
+      <c r="R725" t="str">
+        <v>read</v>
+      </c>
+      <c r="S725" t="str">
+        <v/>
+      </c>
+      <c r="T725" t="str">
+        <v/>
+      </c>
+      <c r="U725" t="str">
+        <v/>
+      </c>
+      <c r="V725">
+        <v>1</v>
+      </c>
+      <c r="W725">
+        <v>0</v>
+      </c>
+      <c r="X725" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y725" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z725" t="str">
+        <v>Literary Fiction</v>
+      </c>
+      <c r="AA725" t="str">
+        <v>Germany</v>
+      </c>
+      <c r="AB725" t="str">
+        <v>German</v>
+      </c>
+      <c r="AC725" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1776505070i/69819.jpg</v>
+      </c>
+      <c r="AD725" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726">
+        <v>12011902</v>
+      </c>
+      <c r="B726" t="str">
+        <v>The Devotion of Suspect X (Detective Galileo, #1)</v>
+      </c>
+      <c r="C726" t="str">
+        <v>Keigo Higashino</v>
+      </c>
+      <c r="D726" t="str">
+        <v>Higashino, Keigo</v>
+      </c>
+      <c r="E726" t="str">
+        <v>Alexander O. Smith</v>
+      </c>
+      <c r="F726" t="str">
+        <v>1250002699</v>
+      </c>
+      <c r="G726" t="str">
+        <v>9781250002693</v>
+      </c>
+      <c r="H726">
+        <v>3</v>
+      </c>
+      <c r="I726" t="str">
+        <v>Minotaur Books</v>
+      </c>
+      <c r="J726" t="str">
+        <v>Paperback</v>
+      </c>
+      <c r="K726">
+        <v>312</v>
+      </c>
+      <c r="L726">
+        <v>2012</v>
+      </c>
+      <c r="M726">
+        <v>2005</v>
+      </c>
+      <c r="N726" s="1" t="d">
+        <v>2026-08-14T00:00:00.000Z</v>
+      </c>
+      <c r="O726" s="1" t="d">
+        <v>2023-02-04T00:00:00.000Z</v>
+      </c>
+      <c r="P726" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q726" t="str">
+        <v>currently-reading (#1), 2026 (#31)</v>
+      </c>
+      <c r="R726" t="str">
+        <v>read</v>
+      </c>
+      <c r="S726" t="str">
+        <v/>
+      </c>
+      <c r="T726" t="str">
+        <v/>
+      </c>
+      <c r="U726" t="str">
+        <v/>
+      </c>
+      <c r="V726">
+        <v>1</v>
+      </c>
+      <c r="W726">
+        <v>0</v>
+      </c>
+      <c r="X726" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y726" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z726" t="str">
+        <v>Crime, Mystery</v>
+      </c>
+      <c r="AA726" t="str">
+        <v>Japan</v>
+      </c>
+      <c r="AB726" t="str">
+        <v>Japanese</v>
+      </c>
+      <c r="AC726" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1495616958i/12011902.jpg</v>
+      </c>
+      <c r="AD726" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727">
+        <v>55077697</v>
+      </c>
+      <c r="B727" t="str">
+        <v>The Blacktongue Thief (Blacktongue, #1)</v>
+      </c>
+      <c r="C727" t="str">
+        <v>Christopher Buehlman</v>
+      </c>
+      <c r="D727" t="str">
+        <v>Buehlman, Christopher</v>
+      </c>
+      <c r="E727" t="str">
+        <v/>
+      </c>
+      <c r="F727" t="str">
+        <v>1250621194</v>
+      </c>
+      <c r="G727" t="str">
+        <v>9781250621191</v>
+      </c>
+      <c r="H727">
+        <v>0</v>
+      </c>
+      <c r="I727" t="str">
+        <v>Tor Books</v>
+      </c>
+      <c r="J727" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K727">
+        <v>416</v>
+      </c>
+      <c r="L727">
+        <v>2021</v>
+      </c>
+      <c r="M727">
+        <v>2021</v>
+      </c>
+      <c r="N727" t="str">
+        <v/>
+      </c>
+      <c r="O727" s="1" t="d">
+        <v>2022-10-16T00:00:00.000Z</v>
+      </c>
+      <c r="P727" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q727" t="str">
+        <v>currently-reading (#1), 2026 (#32)</v>
+      </c>
+      <c r="R727" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S727" t="str">
+        <v/>
+      </c>
+      <c r="T727" t="str">
+        <v/>
+      </c>
+      <c r="U727" t="str">
+        <v/>
+      </c>
+      <c r="V727">
+        <v>1</v>
+      </c>
+      <c r="W727">
+        <v>0</v>
+      </c>
+      <c r="X727" t="str">
+        <v/>
+      </c>
+      <c r="Y727" t="str">
+        <v/>
+      </c>
+      <c r="Z727" t="str">
+        <v/>
+      </c>
+      <c r="AA727" t="str">
+        <v/>
+      </c>
+      <c r="AB727" t="str">
+        <v/>
+      </c>
+      <c r="AC727" t="str">
+        <v>https://covers.openlibrary.org/b/isbn/9781250621191-L.jpg?default=false</v>
+      </c>
+      <c r="AD727" t="str">
+        <v>Claude</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD724"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD727"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
content: import latest Goodreads export, publish Devotion of Suspect X
- Sync Goodreads CSV: The Blacktongue Thief finished (3★), Transcription
  added as a new read, Glorious Exploits now currently-reading
- Fill custom xlsx fields (genre, country, language, gender, cover) for
  the three books; tag Transcription and Outline as Autofiction
- Add draft stub review posts for The Blacktongue Thief and Transcription
- Publish finished review of The Devotion of Suspect X
- Minor recompress of the Savage Detectives post image

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XynQNFFxRcTwwotZTfL3Rn
</commit_message>
<xml_diff>
--- a/book-analysis/website-books.xlsx
+++ b/book-analysis/website-books.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD727"/>
+  <dimension ref="A1:AD729"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -18419,7 +18419,7 @@
         <v>Fiction</v>
       </c>
       <c r="Z196" t="str">
-        <v>Literary Fiction</v>
+        <v>Literary Fiction, Autofiction</v>
       </c>
       <c r="AA196" t="str">
         <v>United Kingdom</v>
@@ -67007,7 +67007,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1342651149i/63033.jpg</v>
       </c>
       <c r="AD724" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="725">
@@ -67191,7 +67191,7 @@
         <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1495616958i/12011902.jpg</v>
       </c>
       <c r="AD726" t="str">
-        <v>Mine</v>
+        <v>Review</v>
       </c>
     </row>
     <row r="727">
@@ -67217,7 +67217,7 @@
         <v>9781250621191</v>
       </c>
       <c r="H727">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I727" t="str">
         <v>Tor Books</v>
@@ -67234,8 +67234,8 @@
       <c r="M727">
         <v>2021</v>
       </c>
-      <c r="N727" t="str">
-        <v/>
+      <c r="N727" s="1" t="d">
+        <v>2026-08-22T00:00:00.000Z</v>
       </c>
       <c r="O727" s="1" t="d">
         <v>2022-10-16T00:00:00.000Z</v>
@@ -67247,7 +67247,7 @@
         <v>currently-reading (#1), 2026 (#32)</v>
       </c>
       <c r="R727" t="str">
-        <v>currently-reading</v>
+        <v>read</v>
       </c>
       <c r="S727" t="str">
         <v/>
@@ -67265,30 +67265,214 @@
         <v>0</v>
       </c>
       <c r="X727" t="str">
-        <v/>
+        <v>Male</v>
       </c>
       <c r="Y727" t="str">
-        <v/>
+        <v>Fiction</v>
       </c>
       <c r="Z727" t="str">
-        <v/>
+        <v>Fantasy</v>
       </c>
       <c r="AA727" t="str">
-        <v/>
+        <v>United States</v>
       </c>
       <c r="AB727" t="str">
-        <v/>
+        <v>English</v>
       </c>
       <c r="AC727" t="str">
-        <v>https://covers.openlibrary.org/b/isbn/9781250621191-L.jpg?default=false</v>
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1604069900i/55077697.jpg</v>
       </c>
       <c r="AD727" t="str">
-        <v>Claude</v>
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728">
+        <v>231387262</v>
+      </c>
+      <c r="B728" t="str">
+        <v>Transcription</v>
+      </c>
+      <c r="C728" t="str">
+        <v>Ben Lerner</v>
+      </c>
+      <c r="D728" t="str">
+        <v>Lerner, Ben</v>
+      </c>
+      <c r="E728" t="str">
+        <v/>
+      </c>
+      <c r="F728" t="str">
+        <v>0374618593</v>
+      </c>
+      <c r="G728" t="str">
+        <v>9780374618599</v>
+      </c>
+      <c r="H728">
+        <v>3</v>
+      </c>
+      <c r="I728" t="str">
+        <v>Farrar, Straus and Giroux</v>
+      </c>
+      <c r="J728" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K728">
+        <v>144</v>
+      </c>
+      <c r="L728">
+        <v>2026</v>
+      </c>
+      <c r="M728">
+        <v>2026</v>
+      </c>
+      <c r="N728" s="1" t="d">
+        <v>2026-08-25T00:00:00.000Z</v>
+      </c>
+      <c r="O728" s="1" t="d">
+        <v>2026-06-06T00:00:00.000Z</v>
+      </c>
+      <c r="P728">
+        <v>2026</v>
+      </c>
+      <c r="Q728" t="str">
+        <v>2026 (#33)</v>
+      </c>
+      <c r="R728" t="str">
+        <v>read</v>
+      </c>
+      <c r="S728" t="str">
+        <v/>
+      </c>
+      <c r="T728" t="str">
+        <v/>
+      </c>
+      <c r="U728" t="str">
+        <v/>
+      </c>
+      <c r="V728">
+        <v>1</v>
+      </c>
+      <c r="W728">
+        <v>0</v>
+      </c>
+      <c r="X728" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y728" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z728" t="str">
+        <v>Literary Fiction, Autofiction</v>
+      </c>
+      <c r="AA728" t="str">
+        <v>United States</v>
+      </c>
+      <c r="AB728" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC728" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1754068063i/231387262.jpg</v>
+      </c>
+      <c r="AD728" t="str">
+        <v>Mine</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729">
+        <v>127278133</v>
+      </c>
+      <c r="B729" t="str">
+        <v>Glorious Exploits</v>
+      </c>
+      <c r="C729" t="str">
+        <v>Ferdia  Lennon</v>
+      </c>
+      <c r="D729" t="str">
+        <v>Lennon, Ferdia</v>
+      </c>
+      <c r="E729" t="str">
+        <v/>
+      </c>
+      <c r="F729" t="str">
+        <v>1250893690</v>
+      </c>
+      <c r="G729" t="str">
+        <v>9781250893697</v>
+      </c>
+      <c r="H729">
+        <v>0</v>
+      </c>
+      <c r="I729" t="str">
+        <v>Henry Holt and Co.</v>
+      </c>
+      <c r="J729" t="str">
+        <v>Hardcover</v>
+      </c>
+      <c r="K729">
+        <v>304</v>
+      </c>
+      <c r="L729">
+        <v>2024</v>
+      </c>
+      <c r="M729">
+        <v>2024</v>
+      </c>
+      <c r="N729" t="str">
+        <v/>
+      </c>
+      <c r="O729" s="1" t="d">
+        <v>2024-11-14T00:00:00.000Z</v>
+      </c>
+      <c r="P729" t="str">
+        <v>currently-reading, 2026</v>
+      </c>
+      <c r="Q729" t="str">
+        <v>currently-reading (#1), 2026 (#34)</v>
+      </c>
+      <c r="R729" t="str">
+        <v>currently-reading</v>
+      </c>
+      <c r="S729" t="str">
+        <v/>
+      </c>
+      <c r="T729" t="str">
+        <v/>
+      </c>
+      <c r="U729" t="str">
+        <v/>
+      </c>
+      <c r="V729">
+        <v>1</v>
+      </c>
+      <c r="W729">
+        <v>0</v>
+      </c>
+      <c r="X729" t="str">
+        <v>Male</v>
+      </c>
+      <c r="Y729" t="str">
+        <v>Fiction</v>
+      </c>
+      <c r="Z729" t="str">
+        <v>Historical Fiction</v>
+      </c>
+      <c r="AA729" t="str">
+        <v>Ireland</v>
+      </c>
+      <c r="AB729" t="str">
+        <v>English</v>
+      </c>
+      <c r="AC729" t="str">
+        <v>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1691418622i/127278133.jpg</v>
+      </c>
+      <c r="AD729" t="str">
+        <v>Mine</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD727"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD729"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>